<commit_message>
add open target and made pipeline services to execute apis
</commit_message>
<xml_diff>
--- a/python_scripts/Cancer_Drugs_MOA.xlsx
+++ b/python_scripts/Cancer_Drugs_MOA.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Drugs &amp; MOA" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Drugs &amp; MOA" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,13 +413,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Drug Name</t>
+          <t>Compound Name</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
@@ -431,7 +431,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>B10</t>
+          <t>Application of Onco-Neutre</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -443,7 +443,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Bevacizumab</t>
+          <t>Application of Onco-Rash</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -455,7 +455,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CT041</t>
+          <t>Epoetin beta</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -467,7 +467,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Drug:</t>
+          <t>Human T Lymphoid Progenitor (HTLP)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -479,39 +479,88 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Etoposide</t>
+          <t>Luveris</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Etoposide inhibits DNA topoisomerase II, thereby inhibiting DNA re-ligation. This causes critical errors in DNA synthesis at the premitotic stage of cell division and can lead to apoptosis of the cancer cell. Etoposide is cell cycle dependent and phase specific, affecting mainly the S and G2 phases of cell division. Inhibition of the topoisomerase II alpha isoform results in the anti-tumour activity of etoposide. The drug is also capable of inhibiting the beta isoform but inhibition of this target is not associated with the anti-tumour activity. It is instead associated with the carcinogenic effect.
-The drug appears to produce its cytotoxic effects by damaging DNA and thereby inhibiting or altering DNA synthesis. ...  Etoposide appears to be cell-cycle dependent and cycle-phase specific, inducing G2 phase arrest and preferentially filling cells in the G2 and late S phases.
-Etoposide has been shown to arrest metaphase in chick fibroblasts, but its principal effect in mammalian cells appears to be in the G2 phase. At etoposide concentrations of 0.3-10 ug/ml in vitro, cells are inhibited from entering prophase; at concentrations of 10 ug/ml or higher, lysis of cells entering mitosis occurs. ... Etoposide does not inhibit microtubule assembly. Etoposide has been shown to induce single-stranded DNA breaks in HeLa cells and in murine leukemia L1210 cells in vitro; the drug also induces double-stranded DNA breaks and DNA-protein crosslinks in L1210 cells. Etoposide induced DNA damage appears to correlate well with the cytotoxicity of the drug. ... Etoposide appears to induce single-stranded DNA breaks indirectly, possibly through endonuclease activation, inhibition of intranuclear type II topoisomerase, or formation of a free-radical metabolite via an enzymatic reaction involving the hydroxyl group at the C-4' position of the E ring. Etoposide also reversibly inhibits the facilitated diffusion of nucleosides into HeLa cells in a concentration dependent manner in vitro.
-Etoposide may stabilize type II topoisomerase DNA complexes, preventing rejoining of single and double strand DNA breaks. Etoposide may also require cellular activation into intermediates, which then bind to DNA and disrupt cellular function.</t>
+          <t>Drug not found in PubChem</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>QL1706</t>
+          <t>Dexrazoxane</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Drug not found in PubChem</t>
+          <t>The mechanism by which dexrazoxane exerts its cardioprotective activity is not fully understood. Dexrazoxane is a cyclic derivative of EDTA that readily penetrates cell membranes. Results of laboratory studies suggest that dexrazoxane (a prodrug) is converted intracellularly to a ring-opened bidentate chelating agent that chelates to free iron and interferes with iron-mediated free radical generation thought to be responsible, in part, for anthracycline-induced cardiomyopathy. It should be noted that dexrazoxane may also be protective through its inhibitory effect on topoisomerase II.
+The mechanism of action of dexrazoxane's cardioprotective activity is not fully understood. Dexrazoxane is a cyclic derivative of ethylenediamine tetra-acetic acid (EDTA) that readily penetrates cell membranes. Laboratory studies suggest that dexrazoxane is converted intracellularly to a ring-opened chelating agent that interferes with iron-mediated free radical generation thought to be responsible, in part, for anthracycline-induced cardiomyopathy.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>XS-03</t>
+          <t>Memantine -Twice Daily or Extended Release</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
           <t>Drug not found in PubChem</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Médialipides</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Drug not found in PubChem</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Smoflipid</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Drug not found in PubChem</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Micafungin</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Micafungin inhibits the synthesis of beta-1,3-D-glucan, an essential component of fungal cell walls which is not present in mammalian cells. It does this by inhibiting beta-1,3-D-glucan synthase.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Sorafenib</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Kinases are involved in tumour cell signalling, proliferation, angiogenesis, and apoptosis. Sorafenib inhibits multiple intracellular serine/threonine kinases in the Ras/mitogen-activated protein kinase (MAPK) signal transduction pathway. Intracellular Raf serine/threonine kinase isoforms inhibited by sorafenib include Raf-1 (or C-Raf), wild-type B-Raf, and mutant B-Raf. Sorafenib inhibits cell surface tyrosine kinase receptors such as KIT, FMS-like tyrosine kinase 3 (FLT-3), RET, RET/PTC, vascular endothelial growth factor receptor-1 (VEGFR-1), VEGFR-2, VEGFR-3, and platelet-derived growth factor receptor-β (PDGFR-β).   Sorafenib is thought to exhibit a dual mechanism of action: it blocks tumour proliferation and growth by inhibiting the RAF/MEK/extracellular signal-regulated kinase (ERK) pathway on tumour cells, and reduces tumour angiogenesis by inhibiting VEGFR and PDGFR signalling in tumour vasculature.
+Sorafenib is U.S. Food and Drug Administration-approved for the treatment of renal cell carcinoma and hepatocellular carcinoma and has been combined with numerous other targeted therapies and chemotherapies in the treatment of many cancers. Unfortunately, as with other RAF inhibitors, patients treated with sorafenib have a 5% to 10% rate of developing cutaneous squamous cell carcinoma (cSCC)/keratoacanthomas. Paradoxical activation of extracellular signal-regulated kinase (ERK) in BRAF wild-type cells has been implicated in RAF inhibitor-induced cSCC. Here, /the researchers/ report that sorafenib suppresses UV-induced apoptosis specifically by inhibiting c-jun-NH2-kinase (JNK) activation through the off-target inhibition of leucine zipper and sterile alpha motif-containing kinase (ZAK). Our results implicate suppression of JNK signaling, independent of the ERK pathway, as an additional mechanism of adverse effects of sorafenib. This has broad implications for combination therapies using sorafenib with other modalities that induce apoptosis.
+Several case reports suggest sorafenib exposure and sorafenib-induced hyperbilirubinemia may be related to a (TA)(5/6/7) repeat polymorphism in UGT1A1*28 (UGT, uridine glucuronosyl transferase). We hypothesized that sorafenib inhibits UGT1A1 and individuals carrying UGT1A1*28 and/or UGT1A9 variants experience greater sorafenib exposure and greater increase in sorafenib-induced plasma bilirubin concentration. Inhibition of UGT1A1-mediated bilirubin glucuronidation by sorafenib was assessed in vitro. UGT1A1*28 and UGT1A9*3 genotypes were ascertained with fragment analysis or direct sequencing in 120 cancer patients receiving sorafenib on five different clinical trials. Total bilirubin measurements were collected in prostate cancer patients before receiving sorafenib (n = 41) and 19 to 30 days following treatment and were compared with UGT1A1*28 genotype. Sorafenib exhibited mixed-mode inhibition of UGT1A1-mediated bilirubin glucuronidation (IC(50) = 18 umol/L; K(i) = 11.7 umol/L) in vitro. Five patients carrying UGT1A1*28/*28 (n = 4) or UGT1A9*3/*3 (n = 1) genotypes had first dose, dose-normalized areas under the sorafenib plasma concentration versus time curve (AUC) that were in the 93rd percentile, whereas three patients carrying UGT1A1*28/*28 had AUCs in the bottom quartile of all genotyped patients. The Drug Metabolizing Enzymes and Transporters genotyping platform was applied to DNA obtained from six patients, which revealed the ABCC2-24C&gt;T genotype cosegregated with sorafenib AUC phenotype. Sorafenib exposure was related to plasma bilirubin increases in patients carrying 1 or 2 copies of UGT1A1*28 alleles (n = 12 and n = 5; R(2) = 0.38 and R(2) = 0.77; P = 0.032 and P = 0.051, respectively). UGT1A1*28 carriers showed two distinct phenotypes that could be explained by ABCC2-24C&gt;T genotype and are more likely to experience plasma bilirubin increases following sorafenib if they had high sorafenib exposure. This pilot study indicates that genotype status of UGT1A1, UGT1A9, and ABCC2 and serum bilirubin concentration increases reflect abnormally high AUC in patients treated with sorafenib.
+Sorafenib is a kinase inhibitor that decreases tumor cell proliferation in vitro.  Sorafenib was shown to inhibit multiple intracellular (c-CRAF, BRAF and mutant BRAF) and cell surface kinases (KIT, FLT- 3, RET, RET/PTC, VEGFR-1, VEGFR- 2, VEGFR- 3, and PDGFR-beta). Several of these kinases are thought to be involved in tumor cell signaling, angiogenesis and apoptosis. Sorafenib inhibited tumor growth of hepatocellular carcinoma (HCC), renal cell carcinoma (RCC), and differentiated thyroid carcinoma (DTC) human tumor xenografts in immunocompromised mice. Reductions in tumor angiogenesis were seen in models of HCC and RCC upon sorafenib treatment, and increases in tumor apoptosis were observed in models of HCC, RCC, and DTC.</t>
         </is>
       </c>
     </row>

</xml_diff>